<commit_message>
update old wss and add unclosed_eq in test
</commit_message>
<xml_diff>
--- a/_other/WeekPlan.xlsx
+++ b/_other/WeekPlan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter2\_other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{762D6B95-7449-467D-91C8-B916FE35BADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81182449-065F-4CEE-998D-85C68C8F6FE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="408">
   <si>
     <t>Новый тест с использованием БД</t>
   </si>
@@ -1261,6 +1261,12 @@
   </si>
   <si>
     <t>Переделать window_test в класс. Добавить такие же возможности, как в RL2.</t>
+  </si>
+  <si>
+    <t>LWS5_EUCLID</t>
+  </si>
+  <si>
+    <t>LWS5_MERCATUS</t>
   </si>
 </sst>
 </file>
@@ -2252,11 +2258,14 @@
       <c r="AL3" s="4" t="s">
         <v>397</v>
       </c>
+      <c r="AM3" s="4" t="s">
+        <v>391</v>
+      </c>
       <c r="AO3" s="2" t="s">
         <v>403</v>
       </c>
       <c r="AP3" s="2" t="s">
-        <v>400</v>
+        <v>392</v>
       </c>
       <c r="AQ3" s="2" t="s">
         <v>382</v>
@@ -2344,11 +2353,11 @@
       <c r="AL4" s="4" t="s">
         <v>393</v>
       </c>
+      <c r="AM4" s="4" t="s">
+        <v>400</v>
+      </c>
       <c r="AO4" s="20" t="s">
         <v>404</v>
-      </c>
-      <c r="AP4" s="2" t="s">
-        <v>391</v>
       </c>
       <c r="AQ4" s="2" t="s">
         <v>384</v>
@@ -2430,9 +2439,6 @@
       <c r="AO5" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="AP5" s="2" t="s">
-        <v>392</v>
-      </c>
       <c r="AQ5" s="2" t="s">
         <v>388</v>
       </c>
@@ -2593,6 +2599,9 @@
       <c r="AL7" s="4" t="s">
         <v>398</v>
       </c>
+      <c r="AM7" s="4" t="s">
+        <v>406</v>
+      </c>
       <c r="AR7" s="2" t="s">
         <v>353</v>
       </c>
@@ -2663,6 +2672,9 @@
       </c>
       <c r="AL8" s="4" t="s">
         <v>401</v>
+      </c>
+      <c r="AM8" s="4" t="s">
+        <v>407</v>
       </c>
       <c r="AR8" s="20" t="s">
         <v>377</v>

</xml_diff>